<commit_message>
Update to Case 1 and Case 2 tests
</commit_message>
<xml_diff>
--- a/Data/PowerWorld/BaselineData/Figure14_22_Baseline.xlsx
+++ b/Data/PowerWorld/BaselineData/Figure14_22_Baseline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\U of Pitt\Spring 2026\Final Project - Distribution Automation\Data\PowerWorld\BaselineData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9466224B-615A-46ED-BEE3-43C9991CF602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B1E5D3-B2CE-47DF-80BC-C5725782EAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4155" yWindow="7620" windowWidth="38700" windowHeight="15345" activeTab="10" xr2:uid="{17303CFB-BDE8-4EBA-829B-F59B3C7383EE}"/>
+    <workbookView xWindow="4185" yWindow="4050" windowWidth="38700" windowHeight="15345" activeTab="2" xr2:uid="{17303CFB-BDE8-4EBA-829B-F59B3C7383EE}"/>
   </bookViews>
   <sheets>
     <sheet name="YBus" sheetId="23" r:id="rId1"/>
@@ -7035,7 +7035,9 @@
   <dimension ref="A1:AC28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="9.140625" style="1"/>
+    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="17.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">

</xml_diff>